<commit_message>
Updates to output locations
1. Output locations updated to ensure each run result is uniquely saved
2. Updated input values for SAF and DACCS filtering for selected studies
3. Updated future fuel price to $1.54/l
</commit_message>
<xml_diff>
--- a/outputs/abatement_cost_curve_SAF.xlsx
+++ b/outputs/abatement_cost_curve_SAF.xlsx
@@ -399,13 +399,13 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>1518.296797214937</v>
+        <v>2338.19769021207</v>
       </c>
       <c r="C2">
-        <v>1025.376992755514</v>
+        <v>1029.089962471334</v>
       </c>
       <c r="D2">
-        <v>3284.240994910336</v>
+        <v>3152.337745755884</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -413,13 +413,13 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>1496.603637338544</v>
+        <v>2279.222732193295</v>
       </c>
       <c r="C3">
-        <v>995.5781210705337</v>
+        <v>987.5291991856195</v>
       </c>
       <c r="D3">
-        <v>3213.22966634006</v>
+        <v>3077.322817063829</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -427,13 +427,13 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>1474.910477462152</v>
+        <v>2220.24777417452</v>
       </c>
       <c r="C4">
-        <v>965.7792493855532</v>
+        <v>945.9684358999053</v>
       </c>
       <c r="D4">
-        <v>3142.218337769784</v>
+        <v>3002.307888371775</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -441,13 +441,13 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>1453.217317585759</v>
+        <v>2161.272816155746</v>
       </c>
       <c r="C5">
-        <v>935.9803777005725</v>
+        <v>904.4076726141913</v>
       </c>
       <c r="D5">
-        <v>3071.207009199508</v>
+        <v>2927.292959679722</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -455,13 +455,13 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>1431.524157709367</v>
+        <v>2102.297858136971</v>
       </c>
       <c r="C6">
-        <v>906.1815060155919</v>
+        <v>862.8469093284772</v>
       </c>
       <c r="D6">
-        <v>3000.195680629232</v>
+        <v>2852.278030987668</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -469,13 +469,13 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>1409.830997832974</v>
+        <v>2043.322900118196</v>
       </c>
       <c r="C7">
-        <v>876.3826343306114</v>
+        <v>821.286146042763</v>
       </c>
       <c r="D7">
-        <v>2929.184352058956</v>
+        <v>2777.263102295613</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -483,13 +483,13 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>1388.137837956581</v>
+        <v>1984.347942099422</v>
       </c>
       <c r="C8">
-        <v>846.5837626456307</v>
+        <v>779.7253827570489</v>
       </c>
       <c r="D8">
-        <v>2858.17302348868</v>
+        <v>2702.248173603559</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -497,13 +497,13 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>1366.444678080189</v>
+        <v>1925.372984080647</v>
       </c>
       <c r="C9">
-        <v>816.7848909606502</v>
+        <v>738.1646194713348</v>
       </c>
       <c r="D9">
-        <v>2787.161694918404</v>
+        <v>2627.233244911505</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -511,13 +511,13 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>1344.751518203796</v>
+        <v>1866.398026061873</v>
       </c>
       <c r="C10">
-        <v>786.9860192756696</v>
+        <v>696.6038561856208</v>
       </c>
       <c r="D10">
-        <v>2716.150366348128</v>
+        <v>2552.218316219451</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -525,13 +525,13 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>1323.058358327403</v>
+        <v>1807.423068043098</v>
       </c>
       <c r="C11">
-        <v>757.1871475906891</v>
+        <v>655.0430928999066</v>
       </c>
       <c r="D11">
-        <v>2645.139037777852</v>
+        <v>2477.203387527397</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -539,13 +539,13 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>1301.365198451011</v>
+        <v>1748.448110024323</v>
       </c>
       <c r="C12">
-        <v>727.3882759057085</v>
+        <v>613.4823296141925</v>
       </c>
       <c r="D12">
-        <v>2574.127709207576</v>
+        <v>2402.188458835343</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -553,13 +553,13 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>1279.672038574618</v>
+        <v>1689.473152005549</v>
       </c>
       <c r="C13">
-        <v>697.5894042207278</v>
+        <v>571.9215663284783</v>
       </c>
       <c r="D13">
-        <v>2503.1163806373</v>
+        <v>2327.173530143289</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -567,13 +567,13 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>1257.978878698226</v>
+        <v>1630.498193986774</v>
       </c>
       <c r="C14">
-        <v>667.7905325357473</v>
+        <v>530.3608030427642</v>
       </c>
       <c r="D14">
-        <v>2432.105052067024</v>
+        <v>2252.158601451235</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -581,13 +581,13 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>1236.285718821833</v>
+        <v>1571.523235967999</v>
       </c>
       <c r="C15">
-        <v>637.9916608507667</v>
+        <v>488.8000397570502</v>
       </c>
       <c r="D15">
-        <v>2361.093723496748</v>
+        <v>2177.143672759181</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -595,13 +595,13 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>1214.59255894544</v>
+        <v>1512.548277949225</v>
       </c>
       <c r="C16">
-        <v>608.1927891657861</v>
+        <v>447.2392764713361</v>
       </c>
       <c r="D16">
-        <v>2290.082394926472</v>
+        <v>2102.128744067127</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -609,13 +609,13 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>1192.899399069048</v>
+        <v>1453.57331993045</v>
       </c>
       <c r="C17">
-        <v>578.3939174808055</v>
+        <v>405.6785131856219</v>
       </c>
       <c r="D17">
-        <v>2219.071066356196</v>
+        <v>2027.113815375073</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -623,13 +623,13 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>1171.206239192655</v>
+        <v>1394.598361911676</v>
       </c>
       <c r="C18">
-        <v>548.5950457958249</v>
+        <v>364.1177498999078</v>
       </c>
       <c r="D18">
-        <v>2148.05973778592</v>
+        <v>1952.098886683019</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -637,13 +637,13 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>1149.513079316263</v>
+        <v>1335.623403892901</v>
       </c>
       <c r="C19">
-        <v>518.7961741108444</v>
+        <v>322.5569866141938</v>
       </c>
       <c r="D19">
-        <v>2077.048409215644</v>
+        <v>1877.083957990965</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -651,13 +651,13 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>1127.81991943987</v>
+        <v>1276.648445874126</v>
       </c>
       <c r="C20">
-        <v>488.9973024258638</v>
+        <v>280.9962233284796</v>
       </c>
       <c r="D20">
-        <v>2006.037080645368</v>
+        <v>1802.069029298911</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -665,13 +665,13 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>1106.126759563477</v>
+        <v>1217.673487855352</v>
       </c>
       <c r="C21">
-        <v>459.1984307408832</v>
+        <v>239.4354600427655</v>
       </c>
       <c r="D21">
-        <v>1935.025752075092</v>
+        <v>1727.054100606857</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -679,13 +679,13 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>1084.433599687085</v>
+        <v>1158.698529836577</v>
       </c>
       <c r="C22">
-        <v>429.3995590559026</v>
+        <v>197.8746967570514</v>
       </c>
       <c r="D22">
-        <v>1864.014423504816</v>
+        <v>1652.039171914803</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -693,13 +693,13 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>1062.740439810692</v>
+        <v>1099.723571817803</v>
       </c>
       <c r="C23">
-        <v>399.6006873709221</v>
+        <v>156.3139334713372</v>
       </c>
       <c r="D23">
-        <v>1793.00309493454</v>
+        <v>1577.024243222749</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -707,13 +707,13 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>1041.047279934299</v>
+        <v>1040.748613799028</v>
       </c>
       <c r="C24">
-        <v>369.8018156859414</v>
+        <v>114.7531701856232</v>
       </c>
       <c r="D24">
-        <v>1721.991766364264</v>
+        <v>1502.009314530695</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -721,13 +721,13 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>1019.354120057907</v>
+        <v>981.7736557802532</v>
       </c>
       <c r="C25">
-        <v>340.0029440009608</v>
+        <v>73.19240689990909</v>
       </c>
       <c r="D25">
-        <v>1650.980437793988</v>
+        <v>1426.994385838641</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -735,13 +735,13 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>997.6609601815142</v>
+        <v>922.7986977614787</v>
       </c>
       <c r="C26">
-        <v>310.2040723159803</v>
+        <v>31.63164361419494</v>
       </c>
       <c r="D26">
-        <v>1579.969109223712</v>
+        <v>1351.979457146587</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updates to save files
1. Updated how savefiles are stored for easier access in plotting code
</commit_message>
<xml_diff>
--- a/outputs/abatement_cost_curve_SAF.xlsx
+++ b/outputs/abatement_cost_curve_SAF.xlsx
@@ -399,7 +399,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>2338.19769021207</v>
+        <v>1430.669687183825</v>
       </c>
       <c r="C2">
         <v>1029.089962471334</v>
@@ -413,13 +413,13 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>2279.222732193295</v>
+        <v>1410.888321154935</v>
       </c>
       <c r="C3">
-        <v>987.5291991856195</v>
+        <v>1004.318977275661</v>
       </c>
       <c r="D3">
-        <v>3077.322817063829</v>
+        <v>3093.385364383004</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -427,13 +427,13 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>2220.24777417452</v>
+        <v>1391.106955126045</v>
       </c>
       <c r="C4">
-        <v>945.9684358999053</v>
+        <v>979.5479920799878</v>
       </c>
       <c r="D4">
-        <v>3002.307888371775</v>
+        <v>3034.432983010125</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -441,13 +441,13 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>2161.272816155746</v>
+        <v>1371.325589097155</v>
       </c>
       <c r="C5">
-        <v>904.4076726141913</v>
+        <v>954.7770068843149</v>
       </c>
       <c r="D5">
-        <v>2927.292959679722</v>
+        <v>2975.480601637246</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -455,13 +455,13 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>2102.297858136971</v>
+        <v>1351.544223068265</v>
       </c>
       <c r="C6">
-        <v>862.8469093284772</v>
+        <v>930.0060216886419</v>
       </c>
       <c r="D6">
-        <v>2852.278030987668</v>
+        <v>2916.528220264366</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -469,13 +469,13 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>2043.322900118196</v>
+        <v>1331.762857039375</v>
       </c>
       <c r="C7">
-        <v>821.286146042763</v>
+        <v>905.235036492969</v>
       </c>
       <c r="D7">
-        <v>2777.263102295613</v>
+        <v>2857.575838891487</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -483,13 +483,13 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>1984.347942099422</v>
+        <v>1311.981491010485</v>
       </c>
       <c r="C8">
-        <v>779.7253827570489</v>
+        <v>880.4640512972961</v>
       </c>
       <c r="D8">
-        <v>2702.248173603559</v>
+        <v>2798.623457518608</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -497,13 +497,13 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>1925.372984080647</v>
+        <v>1292.200124981595</v>
       </c>
       <c r="C9">
-        <v>738.1646194713348</v>
+        <v>855.6930661016232</v>
       </c>
       <c r="D9">
-        <v>2627.233244911505</v>
+        <v>2739.671076145728</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -511,13 +511,13 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>1866.398026061873</v>
+        <v>1272.418758952705</v>
       </c>
       <c r="C10">
-        <v>696.6038561856208</v>
+        <v>830.9220809059503</v>
       </c>
       <c r="D10">
-        <v>2552.218316219451</v>
+        <v>2680.718694772849</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -525,13 +525,13 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>1807.423068043098</v>
+        <v>1252.637392923815</v>
       </c>
       <c r="C11">
-        <v>655.0430928999066</v>
+        <v>806.1510957102773</v>
       </c>
       <c r="D11">
-        <v>2477.203387527397</v>
+        <v>2621.766313399969</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -539,13 +539,13 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>1748.448110024323</v>
+        <v>1232.856026894925</v>
       </c>
       <c r="C12">
-        <v>613.4823296141925</v>
+        <v>781.3801105146044</v>
       </c>
       <c r="D12">
-        <v>2402.188458835343</v>
+        <v>2562.81393202709</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -553,13 +553,13 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>1689.473152005549</v>
+        <v>1213.074660866035</v>
       </c>
       <c r="C13">
-        <v>571.9215663284783</v>
+        <v>756.6091253189315</v>
       </c>
       <c r="D13">
-        <v>2327.173530143289</v>
+        <v>2503.861550654211</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -567,13 +567,13 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>1630.498193986774</v>
+        <v>1193.293294837145</v>
       </c>
       <c r="C14">
-        <v>530.3608030427642</v>
+        <v>731.8381401232587</v>
       </c>
       <c r="D14">
-        <v>2252.158601451235</v>
+        <v>2444.909169281332</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -581,13 +581,13 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>1571.523235967999</v>
+        <v>1173.511928808255</v>
       </c>
       <c r="C15">
-        <v>488.8000397570502</v>
+        <v>707.0671549275858</v>
       </c>
       <c r="D15">
-        <v>2177.143672759181</v>
+        <v>2385.956787908452</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -595,13 +595,13 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>1512.548277949225</v>
+        <v>1153.730562779365</v>
       </c>
       <c r="C16">
-        <v>447.2392764713361</v>
+        <v>682.2961697319129</v>
       </c>
       <c r="D16">
-        <v>2102.128744067127</v>
+        <v>2327.004406535573</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -609,13 +609,13 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>1453.57331993045</v>
+        <v>1133.949196750475</v>
       </c>
       <c r="C17">
-        <v>405.6785131856219</v>
+        <v>657.52518453624</v>
       </c>
       <c r="D17">
-        <v>2027.113815375073</v>
+        <v>2268.052025162694</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -623,13 +623,13 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>1394.598361911676</v>
+        <v>1114.167830721585</v>
       </c>
       <c r="C18">
-        <v>364.1177498999078</v>
+        <v>632.7541993405671</v>
       </c>
       <c r="D18">
-        <v>1952.098886683019</v>
+        <v>2209.099643789814</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -637,13 +637,13 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>1335.623403892901</v>
+        <v>1094.386464692695</v>
       </c>
       <c r="C19">
-        <v>322.5569866141938</v>
+        <v>607.9832141448942</v>
       </c>
       <c r="D19">
-        <v>1877.083957990965</v>
+        <v>2150.147262416935</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -651,13 +651,13 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>1276.648445874126</v>
+        <v>1074.605098663805</v>
       </c>
       <c r="C20">
-        <v>280.9962233284796</v>
+        <v>583.2122289492212</v>
       </c>
       <c r="D20">
-        <v>1802.069029298911</v>
+        <v>2091.194881044056</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -665,13 +665,13 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>1217.673487855352</v>
+        <v>1054.823732634915</v>
       </c>
       <c r="C21">
-        <v>239.4354600427655</v>
+        <v>558.4412437535483</v>
       </c>
       <c r="D21">
-        <v>1727.054100606857</v>
+        <v>2032.242499671176</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -679,13 +679,13 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>1158.698529836577</v>
+        <v>1035.042366606025</v>
       </c>
       <c r="C22">
-        <v>197.8746967570514</v>
+        <v>533.6702585578754</v>
       </c>
       <c r="D22">
-        <v>1652.039171914803</v>
+        <v>1973.290118298297</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -693,13 +693,13 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>1099.723571817803</v>
+        <v>1015.261000577135</v>
       </c>
       <c r="C23">
-        <v>156.3139334713372</v>
+        <v>508.8992733622025</v>
       </c>
       <c r="D23">
-        <v>1577.024243222749</v>
+        <v>1914.337736925418</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -707,13 +707,13 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>1040.748613799028</v>
+        <v>995.4796345482448</v>
       </c>
       <c r="C24">
-        <v>114.7531701856232</v>
+        <v>484.1282881665296</v>
       </c>
       <c r="D24">
-        <v>1502.009314530695</v>
+        <v>1855.385355552538</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -721,13 +721,13 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>981.7736557802532</v>
+        <v>975.6982685193548</v>
       </c>
       <c r="C25">
-        <v>73.19240689990909</v>
+        <v>459.3573029708566</v>
       </c>
       <c r="D25">
-        <v>1426.994385838641</v>
+        <v>1796.432974179659</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -735,13 +735,13 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>922.7986977614787</v>
+        <v>955.9169024904647</v>
       </c>
       <c r="C26">
-        <v>31.63164361419494</v>
+        <v>434.5863177751838</v>
       </c>
       <c r="D26">
-        <v>1351.979457146587</v>
+        <v>1737.48059280678</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixes to contrail abatement sensitivity calculation
</commit_message>
<xml_diff>
--- a/outputs/abatement_cost_curve_SAF.xlsx
+++ b/outputs/abatement_cost_curve_SAF.xlsx
@@ -413,13 +413,13 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>2399.955879687492</v>
+        <v>2378.08102500999</v>
       </c>
       <c r="C3">
-        <v>1038.849562548098</v>
+        <v>1021.863746166218</v>
       </c>
       <c r="D3">
-        <v>3264.448694935819</v>
+        <v>3248.637088882285</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -427,13 +427,13 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>2365.787712548288</v>
+        <v>2322.038003193285</v>
       </c>
       <c r="C4">
-        <v>1013.800071539065</v>
+        <v>979.8284387753048</v>
       </c>
       <c r="D4">
-        <v>3205.431522034906</v>
+        <v>3173.808309927837</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -441,13 +441,13 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>2331.619545409084</v>
+        <v>2265.99498137658</v>
       </c>
       <c r="C5">
-        <v>988.7505805300318</v>
+        <v>937.7931313843915</v>
       </c>
       <c r="D5">
-        <v>3146.414349133992</v>
+        <v>3098.979530973389</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -455,13 +455,13 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>2297.45137826988</v>
+        <v>2209.951959559875</v>
       </c>
       <c r="C6">
-        <v>963.7010895209987</v>
+        <v>895.7578239934783</v>
       </c>
       <c r="D6">
-        <v>3087.397176233078</v>
+        <v>3024.150752018941</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -469,13 +469,13 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>2263.283211130677</v>
+        <v>2153.90893774317</v>
       </c>
       <c r="C7">
-        <v>938.6515985119656</v>
+        <v>853.722516602565</v>
       </c>
       <c r="D7">
-        <v>3028.380003332165</v>
+        <v>2949.321973064493</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -483,13 +483,13 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>2229.115043991473</v>
+        <v>2097.865915926464</v>
       </c>
       <c r="C8">
-        <v>913.6021075029324</v>
+        <v>811.6872092116516</v>
       </c>
       <c r="D8">
-        <v>2969.362830431251</v>
+        <v>2874.493194110045</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -497,13 +497,13 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>2194.94687685227</v>
+        <v>2041.82289410976</v>
       </c>
       <c r="C9">
-        <v>888.5526164938992</v>
+        <v>769.6519018207384</v>
       </c>
       <c r="D9">
-        <v>2910.345657530338</v>
+        <v>2799.664415155597</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -511,13 +511,13 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>2160.778709713066</v>
+        <v>1985.779872293054</v>
       </c>
       <c r="C10">
-        <v>863.5031254848661</v>
+        <v>727.6165944298252</v>
       </c>
       <c r="D10">
-        <v>2851.328484629424</v>
+        <v>2724.835636201149</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -525,13 +525,13 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>2126.610542573862</v>
+        <v>1929.736850476349</v>
       </c>
       <c r="C11">
-        <v>838.453634475833</v>
+        <v>685.5812870389119</v>
       </c>
       <c r="D11">
-        <v>2792.311311728511</v>
+        <v>2650.006857246701</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -539,13 +539,13 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>2092.442375434659</v>
+        <v>1873.693828659644</v>
       </c>
       <c r="C12">
-        <v>813.4041434667998</v>
+        <v>643.5459796479986</v>
       </c>
       <c r="D12">
-        <v>2733.294138827597</v>
+        <v>2575.178078292253</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -553,13 +553,13 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>2058.274208295455</v>
+        <v>1817.650806842939</v>
       </c>
       <c r="C13">
-        <v>788.3546524577666</v>
+        <v>601.5106722570854</v>
       </c>
       <c r="D13">
-        <v>2674.276965926684</v>
+        <v>2500.349299337805</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -567,13 +567,13 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>2024.106041156251</v>
+        <v>1761.607785026234</v>
       </c>
       <c r="C14">
-        <v>763.3051614487335</v>
+        <v>559.4753648661721</v>
       </c>
       <c r="D14">
-        <v>2615.25979302577</v>
+        <v>2425.520520383358</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -581,13 +581,13 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>1989.937874017048</v>
+        <v>1705.564763209529</v>
       </c>
       <c r="C15">
-        <v>738.2556704397005</v>
+        <v>517.4400574752589</v>
       </c>
       <c r="D15">
-        <v>2556.242620124856</v>
+        <v>2350.691741428909</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -595,13 +595,13 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>1955.769706877844</v>
+        <v>1649.521741392824</v>
       </c>
       <c r="C16">
-        <v>713.2061794306672</v>
+        <v>475.4047500843456</v>
       </c>
       <c r="D16">
-        <v>2497.225447223943</v>
+        <v>2275.862962474461</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -609,13 +609,13 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>1921.60153973864</v>
+        <v>1593.478719576119</v>
       </c>
       <c r="C17">
-        <v>688.156688421634</v>
+        <v>433.3694426934323</v>
       </c>
       <c r="D17">
-        <v>2438.208274323029</v>
+        <v>2201.034183520013</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -623,13 +623,13 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>1887.433372599437</v>
+        <v>1537.435697759413</v>
       </c>
       <c r="C18">
-        <v>663.107197412601</v>
+        <v>391.334135302519</v>
       </c>
       <c r="D18">
-        <v>2379.191101422116</v>
+        <v>2126.205404565565</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -637,13 +637,13 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>1853.265205460233</v>
+        <v>1481.392675942709</v>
       </c>
       <c r="C19">
-        <v>638.0577064035679</v>
+        <v>349.2988279116057</v>
       </c>
       <c r="D19">
-        <v>2320.173928521202</v>
+        <v>2051.376625611118</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -651,13 +651,13 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>1819.097038321029</v>
+        <v>1425.349654126003</v>
       </c>
       <c r="C20">
-        <v>613.0082153945347</v>
+        <v>307.2635205206925</v>
       </c>
       <c r="D20">
-        <v>2261.156755620289</v>
+        <v>1976.54784665667</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -665,13 +665,13 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>1784.928871181826</v>
+        <v>1369.306632309298</v>
       </c>
       <c r="C21">
-        <v>587.9587243855015</v>
+        <v>265.2282131297792</v>
       </c>
       <c r="D21">
-        <v>2202.139582719375</v>
+        <v>1901.719067702222</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -679,13 +679,13 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>1750.760704042622</v>
+        <v>1313.263610492593</v>
       </c>
       <c r="C22">
-        <v>562.9092333764684</v>
+        <v>223.192905738866</v>
       </c>
       <c r="D22">
-        <v>2143.122409818462</v>
+        <v>1826.890288747774</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -693,13 +693,13 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>1716.592536903418</v>
+        <v>1257.220588675888</v>
       </c>
       <c r="C23">
-        <v>537.8597423674353</v>
+        <v>181.1575983479527</v>
       </c>
       <c r="D23">
-        <v>2084.105236917548</v>
+        <v>1752.061509793326</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -707,13 +707,13 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>1682.424369764215</v>
+        <v>1201.177566859183</v>
       </c>
       <c r="C24">
-        <v>512.8102513584021</v>
+        <v>139.1222909570395</v>
       </c>
       <c r="D24">
-        <v>2025.088064016634</v>
+        <v>1677.232730838878</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -721,13 +721,13 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>1648.256202625011</v>
+        <v>1145.134545042478</v>
       </c>
       <c r="C25">
-        <v>487.7607603493689</v>
+        <v>97.08698356612615</v>
       </c>
       <c r="D25">
-        <v>1966.070891115721</v>
+        <v>1602.40395188443</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -735,13 +735,13 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>1614.088035485807</v>
+        <v>1089.091523225773</v>
       </c>
       <c r="C26">
-        <v>462.7112693403357</v>
+        <v>55.05167617521291</v>
       </c>
       <c r="D26">
-        <v>1907.053718214807</v>
+        <v>1527.575172929982</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed demand growth rate
</commit_message>
<xml_diff>
--- a/outputs/abatement_cost_curve_SAF.xlsx
+++ b/outputs/abatement_cost_curve_SAF.xlsx
@@ -413,13 +413,13 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>2399.955879687492</v>
+        <v>2398.265833187754</v>
       </c>
       <c r="C3">
-        <v>1038.849562548098</v>
+        <v>1037.221961184374</v>
       </c>
       <c r="D3">
-        <v>3264.448694935819</v>
+        <v>3261.578316510944</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -427,13 +427,13 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>2365.787712548288</v>
+        <v>2362.407619548812</v>
       </c>
       <c r="C4">
-        <v>1013.800071539065</v>
+        <v>1010.544868811617</v>
       </c>
       <c r="D4">
-        <v>3205.431522034906</v>
+        <v>3199.690765185155</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -441,13 +441,13 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>2331.619545409084</v>
+        <v>2326.549405909871</v>
       </c>
       <c r="C5">
-        <v>988.7505805300318</v>
+        <v>983.8677764388597</v>
       </c>
       <c r="D5">
-        <v>3146.414349133992</v>
+        <v>3137.803213859366</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -455,13 +455,13 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>2297.45137826988</v>
+        <v>2290.691192270929</v>
       </c>
       <c r="C6">
-        <v>963.7010895209987</v>
+        <v>957.1906840661023</v>
       </c>
       <c r="D6">
-        <v>3087.397176233078</v>
+        <v>3075.915662533577</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -469,13 +469,13 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>2263.283211130677</v>
+        <v>2254.832978631987</v>
       </c>
       <c r="C7">
-        <v>938.6515985119656</v>
+        <v>930.5135916933451</v>
       </c>
       <c r="D7">
-        <v>3028.380003332165</v>
+        <v>3014.028111207788</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -483,13 +483,13 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>2229.115043991473</v>
+        <v>2218.974764993046</v>
       </c>
       <c r="C8">
-        <v>913.6021075029324</v>
+        <v>903.8364993205879</v>
       </c>
       <c r="D8">
-        <v>2969.362830431251</v>
+        <v>2952.140559881999</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -497,13 +497,13 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>2194.94687685227</v>
+        <v>2183.116551354104</v>
       </c>
       <c r="C9">
-        <v>888.5526164938992</v>
+        <v>877.1594069478307</v>
       </c>
       <c r="D9">
-        <v>2910.345657530338</v>
+        <v>2890.253008556209</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -511,13 +511,13 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>2160.778709713066</v>
+        <v>2147.258337715163</v>
       </c>
       <c r="C10">
-        <v>863.5031254848661</v>
+        <v>850.4823145750735</v>
       </c>
       <c r="D10">
-        <v>2851.328484629424</v>
+        <v>2828.36545723042</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -525,13 +525,13 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>2126.610542573862</v>
+        <v>2111.400124076221</v>
       </c>
       <c r="C11">
-        <v>838.453634475833</v>
+        <v>823.8052222023161</v>
       </c>
       <c r="D11">
-        <v>2792.311311728511</v>
+        <v>2766.477905904631</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -539,13 +539,13 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>2092.442375434659</v>
+        <v>2075.54191043728</v>
       </c>
       <c r="C12">
-        <v>813.4041434667998</v>
+        <v>797.1281298295589</v>
       </c>
       <c r="D12">
-        <v>2733.294138827597</v>
+        <v>2704.590354578842</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -553,13 +553,13 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>2058.274208295455</v>
+        <v>2039.683696798338</v>
       </c>
       <c r="C13">
-        <v>788.3546524577666</v>
+        <v>770.4510374568017</v>
       </c>
       <c r="D13">
-        <v>2674.276965926684</v>
+        <v>2642.702803253053</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -567,13 +567,13 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>2024.106041156251</v>
+        <v>2003.825483159396</v>
       </c>
       <c r="C14">
-        <v>763.3051614487335</v>
+        <v>743.7739450840445</v>
       </c>
       <c r="D14">
-        <v>2615.25979302577</v>
+        <v>2580.815251927264</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -581,13 +581,13 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>1989.937874017048</v>
+        <v>1967.967269520455</v>
       </c>
       <c r="C15">
-        <v>738.2556704397005</v>
+        <v>717.0968527112873</v>
       </c>
       <c r="D15">
-        <v>2556.242620124856</v>
+        <v>2518.927700601475</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -595,13 +595,13 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>1955.769706877844</v>
+        <v>1932.109055881513</v>
       </c>
       <c r="C16">
-        <v>713.2061794306672</v>
+        <v>690.4197603385301</v>
       </c>
       <c r="D16">
-        <v>2497.225447223943</v>
+        <v>2457.040149275686</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -609,13 +609,13 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>1921.60153973864</v>
+        <v>1896.250842242572</v>
       </c>
       <c r="C17">
-        <v>688.156688421634</v>
+        <v>663.7426679657729</v>
       </c>
       <c r="D17">
-        <v>2438.208274323029</v>
+        <v>2395.152597949897</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -623,13 +623,13 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>1887.433372599437</v>
+        <v>1860.39262860363</v>
       </c>
       <c r="C18">
-        <v>663.107197412601</v>
+        <v>637.0655755930156</v>
       </c>
       <c r="D18">
-        <v>2379.191101422116</v>
+        <v>2333.265046624108</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -637,13 +637,13 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>1853.265205460233</v>
+        <v>1824.534414964688</v>
       </c>
       <c r="C19">
-        <v>638.0577064035679</v>
+        <v>610.3884832202584</v>
       </c>
       <c r="D19">
-        <v>2320.173928521202</v>
+        <v>2271.377495298319</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -651,13 +651,13 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>1819.097038321029</v>
+        <v>1788.676201325747</v>
       </c>
       <c r="C20">
-        <v>613.0082153945347</v>
+        <v>583.7113908475011</v>
       </c>
       <c r="D20">
-        <v>2261.156755620289</v>
+        <v>2209.48994397253</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -665,13 +665,13 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>1784.928871181826</v>
+        <v>1752.817987686805</v>
       </c>
       <c r="C21">
-        <v>587.9587243855015</v>
+        <v>557.0342984747439</v>
       </c>
       <c r="D21">
-        <v>2202.139582719375</v>
+        <v>2147.602392646741</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -679,13 +679,13 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>1750.760704042622</v>
+        <v>1716.959774047864</v>
       </c>
       <c r="C22">
-        <v>562.9092333764684</v>
+        <v>530.3572061019867</v>
       </c>
       <c r="D22">
-        <v>2143.122409818462</v>
+        <v>2085.714841320952</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -693,13 +693,13 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>1716.592536903418</v>
+        <v>1681.101560408922</v>
       </c>
       <c r="C23">
-        <v>537.8597423674353</v>
+        <v>503.6801137292294</v>
       </c>
       <c r="D23">
-        <v>2084.105236917548</v>
+        <v>2023.827289995163</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -707,13 +707,13 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>1682.424369764215</v>
+        <v>1645.243346769981</v>
       </c>
       <c r="C24">
-        <v>512.8102513584021</v>
+        <v>477.0030213564722</v>
       </c>
       <c r="D24">
-        <v>2025.088064016634</v>
+        <v>1961.939738669374</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -721,13 +721,13 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>1648.256202625011</v>
+        <v>1609.385133131039</v>
       </c>
       <c r="C25">
-        <v>487.7607603493689</v>
+        <v>450.3259289837149</v>
       </c>
       <c r="D25">
-        <v>1966.070891115721</v>
+        <v>1900.052187343585</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -735,13 +735,13 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>1614.088035485807</v>
+        <v>1573.526919492097</v>
       </c>
       <c r="C26">
-        <v>462.7112693403357</v>
+        <v>423.6488366109576</v>
       </c>
       <c r="D26">
-        <v>1907.053718214807</v>
+        <v>1838.164636017796</v>
       </c>
     </row>
   </sheetData>

</xml_diff>